<commit_message>
feat(employee): add gender support and homepage carousel updates
</commit_message>
<xml_diff>
--- a/backend/StoreManagementService/docs/employee-migration/employee_migration_template.xlsx
+++ b/backend/StoreManagementService/docs/employee-migration/employee_migration_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>emp_id</t>
   </si>
@@ -38,6 +38,9 @@
     <t>group_head</t>
   </si>
   <si>
+    <t>gender</t>
+  </si>
+  <si>
     <t>office_location</t>
   </si>
   <si>
@@ -62,6 +65,9 @@
     <t>Rohit Sharma</t>
   </si>
   <si>
+    <t>Male</t>
+  </si>
+  <si>
     <t>Panchkula</t>
   </si>
   <si>
@@ -86,6 +92,9 @@
     <t>Anil Gupta</t>
   </si>
   <si>
+    <t>Female</t>
+  </si>
+  <si>
     <t>Chandigarh</t>
   </si>
   <si>
@@ -95,10 +104,16 @@
     <t>Fill data in 'employees' sheet only. Do not change header names.</t>
   </si>
   <si>
-    <t>Required columns: emp_id, name, father_name, email_id, mobile_no, designation, division, group_head, office_location.</t>
+    <t>Required columns: emp_id, name, father_name, email_id, mobile_no, designation, division, group_head, gender, office_location.</t>
+  </si>
+  <si>
+    <t>Allowed values for gender: Male, Female, Other.</t>
   </si>
   <si>
     <t>emp_id must be a positive integer. mobile_no must be 10 digits and start with 6-9.</t>
+  </si>
+  <si>
+    <t>office_location drives location-aware access, requisitions, stock issue, and migration routing. Use the exact location names used in Access Control, for example Panchkula.</t>
   </si>
   <si>
     <t>Use validate API first, then execute API.</t>
@@ -482,14 +497,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="8" width="16" customWidth="1"/>
-    <col min="9" max="9" width="19" customWidth="1"/>
+    <col min="1" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -517,63 +532,72 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>101</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="E2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+      <c r="J2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>102</v>
       </c>
       <c r="B3" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C3" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D3" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="G3" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H3" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I3" t="s">
-        <v>24</v>
+        <v>26</v>
+      </c>
+      <c r="J3" t="s">
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -584,7 +608,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A5"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="120" customWidth="1"/>
@@ -592,27 +616,37 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
refactor(employee): remove group head from store employee flow
</commit_message>
<xml_diff>
--- a/backend/StoreManagementService/docs/employee-migration/employee_migration_template.xlsx
+++ b/backend/StoreManagementService/docs/employee-migration/employee_migration_template.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>emp_id</t>
   </si>
@@ -35,9 +35,6 @@
     <t>division</t>
   </si>
   <si>
-    <t>group_head</t>
-  </si>
-  <si>
     <t>gender</t>
   </si>
   <si>
@@ -62,9 +59,6 @@
     <t>Procurement</t>
   </si>
   <si>
-    <t>Rohit Sharma</t>
-  </si>
-  <si>
     <t>Male</t>
   </si>
   <si>
@@ -89,9 +83,6 @@
     <t>Admin</t>
   </si>
   <si>
-    <t>Anil Gupta</t>
-  </si>
-  <si>
     <t>Female</t>
   </si>
   <si>
@@ -104,7 +95,7 @@
     <t>Fill data in 'employees' sheet only. Do not change header names.</t>
   </si>
   <si>
-    <t>Required columns: emp_id, name, father_name, email_id, mobile_no, designation, division, group_head, gender, office_location.</t>
+    <t>Required columns: emp_id, name, father_name, email_id, mobile_no, designation, division, gender, office_location.</t>
   </si>
   <si>
     <t>Allowed values for gender: Male, Female, Other.</t>
@@ -497,14 +488,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="9" width="16" customWidth="1"/>
-    <col min="10" max="10" width="19" customWidth="1"/>
+    <col min="1" max="8" width="16" customWidth="1"/>
+    <col min="9" max="9" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -532,72 +523,63 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>101</v>
       </c>
       <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>12</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>14</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>15</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>16</v>
       </c>
-      <c r="I2" t="s">
-        <v>17</v>
-      </c>
-      <c r="J2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>102</v>
       </c>
       <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
         <v>19</v>
       </c>
-      <c r="C3" t="s">
+      <c r="E3" t="s">
         <v>20</v>
       </c>
-      <c r="D3" t="s">
+      <c r="F3" t="s">
         <v>21</v>
       </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>22</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>23</v>
       </c>
-      <c r="G3" t="s">
+      <c r="I3" t="s">
         <v>24</v>
-      </c>
-      <c r="H3" t="s">
-        <v>25</v>
-      </c>
-      <c r="I3" t="s">
-        <v>26</v>
-      </c>
-      <c r="J3" t="s">
-        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -616,37 +598,37 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>